<commit_message>
Bổ sung Luật 93/2025/QH15, sơ đồ và điều chỉnh nội dung 3 chương theo góp ý
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ThGArqDrUUsqC1zG1BQvVL
</commit_message>
<xml_diff>
--- a/Ban_cuoi/Du_lieu_bieu_do_Chuong_2.xlsx
+++ b/Ban_cuoi/Du_lieu_bieu_do_Chuong_2.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Muc_luc" sheetId="1" r:id="rId1"/>
     <sheet name="H2.1" sheetId="2" r:id="rId2"/>
     <sheet name="H2.2" sheetId="3" r:id="rId3"/>
-    <sheet name="H2.3" sheetId="4" r:id="rId4"/>
-    <sheet name="H2.4" sheetId="5" r:id="rId5"/>
-    <sheet name="H2.5" sheetId="6" r:id="rId6"/>
-    <sheet name="H2.6" sheetId="7" r:id="rId7"/>
-    <sheet name="H2.7" sheetId="8" r:id="rId8"/>
-    <sheet name="H2.8" sheetId="9" r:id="rId9"/>
-    <sheet name="H2.9" sheetId="10" r:id="rId10"/>
+    <sheet name="H2.4" sheetId="4" r:id="rId4"/>
+    <sheet name="H2.5" sheetId="5" r:id="rId5"/>
+    <sheet name="H2.6" sheetId="6" r:id="rId6"/>
+    <sheet name="H2.7" sheetId="7" r:id="rId7"/>
+    <sheet name="H2.8" sheetId="8" r:id="rId8"/>
+    <sheet name="H2.9" sheetId="9" r:id="rId9"/>
+    <sheet name="H2.10" sheetId="10" r:id="rId10"/>
     <sheet name="Nhat_ky_chuan_hoa" sheetId="11" r:id="rId11"/>
     <sheet name="DL_De_tai" sheetId="12" r:id="rId12"/>
     <sheet name="DL_TSTT" sheetId="13" r:id="rId13"/>
@@ -62,67 +62,67 @@
     <t>H2.2</t>
   </si>
   <si>
-    <t>Hình 2.3</t>
+    <t>Hình 2.4</t>
   </si>
   <si>
     <t>Số đề tài cấp cơ sở theo hình thức kinh phí và kinh phí Nhà trường cấp, giai đoạn 2021 - 2025</t>
   </si>
   <si>
-    <t>H2.3</t>
-  </si>
-  <si>
-    <t>Hình 2.4</t>
+    <t>H2.4</t>
+  </si>
+  <si>
+    <t>Hình 2.5</t>
   </si>
   <si>
     <t>Giờ nghiên cứu quy đổi và mức thưởng bằng tiền theo loại sản phẩm khoa học</t>
   </si>
   <si>
-    <t>H2.4</t>
-  </si>
-  <si>
-    <t>Hình 2.5</t>
+    <t>H2.5</t>
+  </si>
+  <si>
+    <t>Hình 2.6</t>
   </si>
   <si>
     <t>Khả năng tính toán bộ tiêu chí đánh giá hiệu quả quản lý quyền sở hữu trí tuệ từ dữ liệu hiện có</t>
   </si>
   <si>
-    <t>H2.5</t>
-  </si>
-  <si>
-    <t>Hình 2.6</t>
+    <t>H2.6</t>
+  </si>
+  <si>
+    <t>Hình 2.7</t>
   </si>
   <si>
     <t>Tài sản trí tuệ của Nhà trường theo loại hình và tình trạng pháp lý</t>
   </si>
   <si>
-    <t>H2.6</t>
-  </si>
-  <si>
-    <t>Hình 2.7</t>
+    <t>H2.7</t>
+  </si>
+  <si>
+    <t>Hình 2.8</t>
   </si>
   <si>
     <t>Sản phẩm đề tài cấp cơ sở đủ điều kiện xác lập quyền theo nhóm quyền có thể xác lập</t>
   </si>
   <si>
-    <t>H2.7</t>
-  </si>
-  <si>
-    <t>Hình 2.8</t>
+    <t>H2.8</t>
+  </si>
+  <si>
+    <t>Hình 2.9</t>
   </si>
   <si>
     <t>Chuỗi chuyển hóa từ đề tài cấp cơ sở sang đơn đăng ký sở hữu công nghiệp</t>
   </si>
   <si>
-    <t>H2.8</t>
-  </si>
-  <si>
-    <t>Hình 2.9</t>
+    <t>H2.9</t>
+  </si>
+  <si>
+    <t>Hình 2.10</t>
   </si>
   <si>
     <t>Tỷ lệ thực hiện so với chỉ tiêu Kế hoạch 07/KH-ĐHTĐ, cộng dồn hai năm 2024 - 2025</t>
   </si>
   <si>
-    <t>H2.9</t>
+    <t>H2.10</t>
   </si>
   <si>
     <t>Các chỉnh sửa số liệu so với bản Chương 2 trước</t>
@@ -200,7 +200,7 @@
     <t>Hình 2.2. Mô phỏng phần lợi ích của tác giả theo các quy định nội bộ và mức mặc định của Luật Sở hữu trí tuệ</t>
   </si>
   <si>
-    <t>Nguồn: Nhóm nghiên cứu mô phỏng từ Điều 36 Quyết định 213, Điều 9 Điều lệ Quỹ Học bổng sau tiến sĩ Ngô Xuân Độ và điểm b khoản 1 Điều 135 Luật Sở hữu trí tuệ. Khoản thu là số tiền nhận được từ một hợp đồng chuyển giao sau khi trừ chi phí hợp lệ; đơn vị: triệu đồng.</t>
+    <t>Nguồn: Nhóm nghiên cứu mô phỏng từ Điều 36 Quyết định 213, Điều 9 Điều lệ Quỹ Học bổng sau tiến sĩ Ngô Xuân Độ, điểm b khoản 1 Điều 135 Luật Sở hữu trí tuệ và điểm a khoản 3 Điều 28 Luật số 93/2025/QH15. Khoản thu là số tiền nhận được từ một hợp đồng chuyển giao sau khi trừ chi phí hợp lệ; đơn vị: triệu đồng.</t>
   </si>
   <si>
     <t>Khoản thu từ chuyển giao</t>
@@ -245,7 +245,7 @@
     <t>700</t>
   </si>
   <si>
-    <t>Hình 2.3. Số đề tài cấp cơ sở theo hình thức kinh phí và kinh phí Nhà trường cấp, giai đoạn 2021 - 2025</t>
+    <t>Hình 2.4. Số đề tài cấp cơ sở theo hình thức kinh phí và kinh phí Nhà trường cấp, giai đoạn 2021 - 2025</t>
   </si>
   <si>
     <t>Nguồn: Nhóm nghiên cứu tổng hợp từ danh mục đề tài khoa học công nghệ cấp cơ sở giai đoạn 2021 - 2025. Đề tài xếp theo năm ghi trong mã số; kinh phí đơn vị triệu đồng.</t>
@@ -263,7 +263,7 @@
     <t>Kinh phí Nhà trường cấp (triệu đồng)</t>
   </si>
   <si>
-    <t>Hình 2.4. Giờ nghiên cứu quy đổi và mức thưởng bằng tiền theo loại sản phẩm khoa học</t>
+    <t>Hình 2.5. Giờ nghiên cứu quy đổi và mức thưởng bằng tiền theo loại sản phẩm khoa học</t>
   </si>
   <si>
     <t>Nguồn: Nhóm nghiên cứu tổng hợp từ Bảng 6 và Bảng 7, Quy chế chi tiêu nội bộ Trường Đại học Thành Đô ban hành ngày 01 tháng 8 năm 2026. Sáng chế chuẩn quốc tế là bằng độc quyền theo chuẩn Mỹ, châu Âu, Đông Bắc Á; sáng chế chuẩn Việt Nam là bằng độc quyền theo chuẩn Việt Nam, Trung Quốc, ASEAN. Mức thưởng là tổng tiền thưởng cho một bài báo.</t>
@@ -302,7 +302,7 @@
     <t>Bài trong nước 1,75 điểm</t>
   </si>
   <si>
-    <t>Hình 2.5. Khả năng tính toán bộ tiêu chí đánh giá hiệu quả quản lý quyền sở hữu trí tuệ từ dữ liệu hiện có</t>
+    <t>Hình 2.6. Khả năng tính toán bộ tiêu chí đánh giá hiệu quả quản lý quyền sở hữu trí tuệ từ dữ liệu hiện có</t>
   </si>
   <si>
     <t>Nguồn: Đánh giá của nhóm nghiên cứu đối với 16 tiêu chí tại Mục 1.4.2, căn cứ vào các danh mục và văn bản hiện có của Trường Đại học Thành Đô. Chi tiết từng tiêu chí tại tệp dữ liệu kèm theo.</t>
@@ -332,7 +332,7 @@
     <t>Kết quả</t>
   </si>
   <si>
-    <t>Hình 2.6. Tài sản trí tuệ của Nhà trường theo loại hình và tình trạng pháp lý</t>
+    <t>Hình 2.7. Tài sản trí tuệ của Nhà trường theo loại hình và tình trạng pháp lý</t>
   </si>
   <si>
     <t>Nguồn: Nhóm nghiên cứu tổng hợp từ Bảng 2.6.</t>
@@ -362,7 +362,7 @@
     <t>Sáng chế</t>
   </si>
   <si>
-    <t>Hình 2.7. Sản phẩm đề tài cấp cơ sở đủ điều kiện xác lập quyền theo nhóm quyền có thể xác lập</t>
+    <t>Hình 2.8. Sản phẩm đề tài cấp cơ sở đủ điều kiện xác lập quyền theo nhóm quyền có thể xác lập</t>
   </si>
   <si>
     <t>Nguồn: Nhóm nghiên cứu tổng hợp từ Bảng 2.7.</t>
@@ -383,7 +383,7 @@
     <t>Kiểu dáng công nghiệp hoặc giải pháp hữu ích</t>
   </si>
   <si>
-    <t>Hình 2.8. Chuỗi chuyển hóa từ đề tài cấp cơ sở sang đơn đăng ký sở hữu công nghiệp</t>
+    <t>Hình 2.9. Chuỗi chuyển hóa từ đề tài cấp cơ sở sang đơn đăng ký sở hữu công nghiệp</t>
   </si>
   <si>
     <t>Nguồn: Nhóm nghiên cứu tính toán từ danh mục đề tài cấp cơ sở và Bảng 2.7.</t>
@@ -407,7 +407,7 @@
     <t>Đã nộp đơn đăng ký</t>
   </si>
   <si>
-    <t>Hình 2.9. Tỷ lệ thực hiện so với chỉ tiêu Kế hoạch 07/KH-ĐHTĐ, cộng dồn hai năm 2024 - 2025</t>
+    <t>Hình 2.10. Tỷ lệ thực hiện so với chỉ tiêu Kế hoạch 07/KH-ĐHTĐ, cộng dồn hai năm 2024 - 2025</t>
   </si>
   <si>
     <t>Nguồn: Nhóm nghiên cứu tính toán từ mục 2.2.4 Kế hoạch số 07/KH-ĐHTĐ ngày 01 tháng 7 năm 2024 và các danh mục thống kê của Phòng Khoa học Công nghệ. Chỉ tiêu bài báo trong nước gồm bài đăng tạp chí trong nước và tạp chí của Trường; văn bằng sở hữu trí tuệ gồm sáng chế, kiểu dáng công nghiệp, quyền tác giả được cấp; không gồm tham luận hội thảo quốc gia do danh mục không có năm. Màu xanh dương: công bố; xanh lục: đề tài và học liệu; cam: tài sản trí tuệ.</t>
@@ -2977,7 +2977,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.3'!$B$4</c:f>
+              <c:f>'H2.4'!$B$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2998,7 +2998,7 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>'H2.3'!$A$5:$A$9</c:f>
+              <c:f>'H2.4'!$A$5:$A$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3022,7 +3022,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.3'!$B$5:$B$9</c:f>
+              <c:f>'H2.4'!$B$5:$B$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3050,7 +3050,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.3'!$C$4</c:f>
+              <c:f>'H2.4'!$C$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3071,7 +3071,7 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>'H2.3'!$A$5:$A$9</c:f>
+              <c:f>'H2.4'!$A$5:$A$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3095,7 +3095,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.3'!$C$5:$C$9</c:f>
+              <c:f>'H2.4'!$C$5:$C$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3123,7 +3123,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.3'!$D$4</c:f>
+              <c:f>'H2.4'!$D$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3144,7 +3144,7 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>'H2.3'!$A$5:$A$9</c:f>
+              <c:f>'H2.4'!$A$5:$A$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3168,7 +3168,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.3'!$D$5:$D$9</c:f>
+              <c:f>'H2.4'!$D$5:$D$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3203,7 +3203,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.3'!$E$4</c:f>
+              <c:f>'H2.4'!$E$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3264,7 +3264,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>'H2.3'!$A$5:$A$9</c:f>
+              <c:f>'H2.4'!$A$5:$A$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3288,7 +3288,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.3'!$E$5:$E$9</c:f>
+              <c:f>'H2.4'!$E$5:$E$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3586,7 +3586,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.4'!$B$4</c:f>
+              <c:f>'H2.5'!$B$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3735,7 +3735,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.4'!$A$5:$A$12</c:f>
+              <c:f>'H2.5'!$A$5:$A$12</c:f>
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
@@ -3767,7 +3767,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.4'!$B$5:$B$12</c:f>
+              <c:f>'H2.5'!$B$5:$B$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -3810,7 +3810,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.4'!$C$4</c:f>
+              <c:f>'H2.5'!$C$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3881,7 +3881,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.4'!$A$5:$A$12</c:f>
+              <c:f>'H2.5'!$A$5:$A$12</c:f>
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
@@ -3913,7 +3913,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.4'!$C$5:$C$12</c:f>
+              <c:f>'H2.5'!$C$5:$C$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -4220,7 +4220,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.5'!$B$4</c:f>
+              <c:f>'H2.6'!$B$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4270,7 +4270,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.5'!$A$5:$A$8</c:f>
+              <c:f>'H2.6'!$A$5:$A$8</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -4290,7 +4290,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.5'!$B$5:$B$8</c:f>
+              <c:f>'H2.6'!$B$5:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -4315,7 +4315,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.5'!$C$4</c:f>
+              <c:f>'H2.6'!$C$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4361,7 +4361,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.5'!$A$5:$A$8</c:f>
+              <c:f>'H2.6'!$A$5:$A$8</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -4381,7 +4381,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.5'!$C$5:$C$8</c:f>
+              <c:f>'H2.6'!$C$5:$C$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -4406,7 +4406,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.5'!$D$4</c:f>
+              <c:f>'H2.6'!$D$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4456,7 +4456,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.5'!$A$5:$A$8</c:f>
+              <c:f>'H2.6'!$A$5:$A$8</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -4476,7 +4476,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.5'!$D$5:$D$8</c:f>
+              <c:f>'H2.6'!$D$5:$D$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -4690,7 +4690,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.6'!$B$4</c:f>
+              <c:f>'H2.7'!$B$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4740,7 +4740,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.6'!$A$5:$A$8</c:f>
+              <c:f>'H2.7'!$A$5:$A$8</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -4760,7 +4760,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.6'!$B$5:$B$8</c:f>
+              <c:f>'H2.7'!$B$5:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -4785,7 +4785,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.6'!$C$4</c:f>
+              <c:f>'H2.7'!$C$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4839,7 +4839,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.6'!$A$5:$A$8</c:f>
+              <c:f>'H2.7'!$A$5:$A$8</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -4859,7 +4859,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.6'!$C$5:$C$8</c:f>
+              <c:f>'H2.7'!$C$5:$C$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -5073,7 +5073,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.7'!$B$4</c:f>
+              <c:f>'H2.8'!$B$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5183,7 +5183,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.7'!$A$5:$A$9</c:f>
+              <c:f>'H2.8'!$A$5:$A$9</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -5206,7 +5206,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.7'!$B$5:$B$9</c:f>
+              <c:f>'H2.8'!$B$5:$B$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -5394,7 +5394,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.8'!$B$4</c:f>
+              <c:f>'H2.9'!$B$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5439,7 +5439,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.8'!$A$5:$A$7</c:f>
+              <c:f>'H2.9'!$A$5:$A$7</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -5456,7 +5456,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.8'!$B$5:$B$7</c:f>
+              <c:f>'H2.9'!$B$5:$B$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -5478,7 +5478,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.8'!$C$4</c:f>
+              <c:f>'H2.9'!$C$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5523,7 +5523,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.8'!$A$5:$A$7</c:f>
+              <c:f>'H2.9'!$A$5:$A$7</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -5540,7 +5540,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.8'!$C$5:$C$7</c:f>
+              <c:f>'H2.9'!$C$5:$C$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -5750,7 +5750,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'H2.9'!$E$4</c:f>
+              <c:f>'H2.10'!$E$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5925,7 +5925,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'H2.9'!$A$5:$A$14</c:f>
+              <c:f>'H2.10'!$A$5:$A$14</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -5963,7 +5963,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'H2.9'!$E$5:$E$14</c:f>
+              <c:f>'H2.10'!$E$5:$E$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -6905,13 +6905,13 @@
   <hyperlinks>
     <hyperlink ref="C5" location="'H2.1'!A1" display="H2.1"/>
     <hyperlink ref="C6" location="'H2.2'!A1" display="H2.2"/>
-    <hyperlink ref="C7" location="'H2.3'!A1" display="H2.3"/>
-    <hyperlink ref="C8" location="'H2.4'!A1" display="H2.4"/>
-    <hyperlink ref="C9" location="'H2.5'!A1" display="H2.5"/>
-    <hyperlink ref="C10" location="'H2.6'!A1" display="H2.6"/>
-    <hyperlink ref="C11" location="'H2.7'!A1" display="H2.7"/>
-    <hyperlink ref="C12" location="'H2.8'!A1" display="H2.8"/>
-    <hyperlink ref="C13" location="'H2.9'!A1" display="H2.9"/>
+    <hyperlink ref="C7" location="'H2.4'!A1" display="H2.4"/>
+    <hyperlink ref="C8" location="'H2.5'!A1" display="H2.5"/>
+    <hyperlink ref="C9" location="'H2.6'!A1" display="H2.6"/>
+    <hyperlink ref="C10" location="'H2.7'!A1" display="H2.7"/>
+    <hyperlink ref="C11" location="'H2.8'!A1" display="H2.8"/>
+    <hyperlink ref="C12" location="'H2.9'!A1" display="H2.9"/>
+    <hyperlink ref="C13" location="'H2.10'!A1" display="H2.10"/>
     <hyperlink ref="C15" location="'Nhat_ky_chuan_hoa'!A1" display="Nhat_ky_chuan_hoa"/>
     <hyperlink ref="C16" location="'DL_De_tai'!A1" display="DL_De_tai"/>
     <hyperlink ref="C17" location="'DL_TSTT'!A1" display="DL_TSTT"/>

</xml_diff>